<commit_message>
docs: enhance performance analysis section with detailed throughput and latency insights
</commit_message>
<xml_diff>
--- a/Results/charts/stats.xlsx
+++ b/Results/charts/stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\progetti_uni\sistemi_architetture_bd\proj_stream\Results\charts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{778BB6C2-D04E-46F9-B023-24316AEA7270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19B22E30-444E-4ADA-B29F-1BC4D9263AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{C00845A1-E4B8-49E1-B98B-5AC65EED64DF}"/>
   </bookViews>
@@ -1051,26 +1051,66 @@
       <c r="A12" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="8"/>
-      <c r="N12" s="8"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="8"/>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="8"/>
-      <c r="S12" s="8"/>
-      <c r="T12" s="8"/>
-      <c r="U12" s="8"/>
+      <c r="B12" s="7">
+        <v>2730</v>
+      </c>
+      <c r="C12" s="8">
+        <v>646</v>
+      </c>
+      <c r="D12" s="8">
+        <v>92.1</v>
+      </c>
+      <c r="E12" s="8">
+        <v>21.9</v>
+      </c>
+      <c r="F12" s="8">
+        <v>12</v>
+      </c>
+      <c r="G12" s="8">
+        <v>2.75</v>
+      </c>
+      <c r="H12" s="8">
+        <v>54.4</v>
+      </c>
+      <c r="I12" s="8">
+        <v>12.8</v>
+      </c>
+      <c r="J12" s="8">
+        <v>26.1</v>
+      </c>
+      <c r="K12" s="9">
+        <v>5.87</v>
+      </c>
+      <c r="L12" s="7">
+        <v>2950</v>
+      </c>
+      <c r="M12" s="8">
+        <v>243</v>
+      </c>
+      <c r="N12" s="8">
+        <v>99.6</v>
+      </c>
+      <c r="O12" s="8">
+        <v>6.61</v>
+      </c>
+      <c r="P12" s="8">
+        <v>12.9</v>
+      </c>
+      <c r="Q12" s="8">
+        <v>0.61199999999999999</v>
+      </c>
+      <c r="R12" s="8">
+        <v>58.7</v>
+      </c>
+      <c r="S12" s="8">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="T12" s="8">
+        <v>28</v>
+      </c>
+      <c r="U12" s="8">
+        <v>2.0099999999999998</v>
+      </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
@@ -1254,26 +1294,66 @@
       <c r="A17" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="9"/>
-      <c r="L17" s="7"/>
-      <c r="M17" s="8"/>
-      <c r="N17" s="8"/>
-      <c r="O17" s="8"/>
-      <c r="P17" s="8"/>
-      <c r="Q17" s="8"/>
-      <c r="R17" s="8"/>
-      <c r="S17" s="8"/>
-      <c r="T17" s="8"/>
-      <c r="U17" s="8"/>
+      <c r="B17" s="7">
+        <v>2780</v>
+      </c>
+      <c r="C17" s="8">
+        <v>596</v>
+      </c>
+      <c r="D17" s="8">
+        <v>94.5</v>
+      </c>
+      <c r="E17" s="8">
+        <v>20.3</v>
+      </c>
+      <c r="F17" s="8">
+        <v>12.2</v>
+      </c>
+      <c r="G17" s="8">
+        <v>2.48</v>
+      </c>
+      <c r="H17" s="8">
+        <v>56</v>
+      </c>
+      <c r="I17" s="8">
+        <v>12.1</v>
+      </c>
+      <c r="J17" s="8">
+        <v>26.2</v>
+      </c>
+      <c r="K17" s="9">
+        <v>5.94</v>
+      </c>
+      <c r="L17" s="7">
+        <v>2980</v>
+      </c>
+      <c r="M17" s="8">
+        <v>160</v>
+      </c>
+      <c r="N17" s="8">
+        <v>102</v>
+      </c>
+      <c r="O17" s="8">
+        <v>2.73</v>
+      </c>
+      <c r="P17" s="8">
+        <v>13.1</v>
+      </c>
+      <c r="Q17" s="8">
+        <v>0.128</v>
+      </c>
+      <c r="R17" s="8">
+        <v>60.2</v>
+      </c>
+      <c r="S17" s="8">
+        <v>2.4</v>
+      </c>
+      <c r="T17" s="8">
+        <v>28.3</v>
+      </c>
+      <c r="U17" s="8">
+        <v>1.28</v>
+      </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="5"/>

</xml_diff>

<commit_message>
docs: update throughput statistics tables for improved clarity and consistency
</commit_message>
<xml_diff>
--- a/Results/charts/stats.xlsx
+++ b/Results/charts/stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\progetti_uni\sistemi_architetture_bd\proj_stream\Results\charts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19B22E30-444E-4ADA-B29F-1BC4D9263AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC0A5B92-A8F8-4E69-909D-3F5AA5EA01AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{C00845A1-E4B8-49E1-B98B-5AC65EED64DF}"/>
   </bookViews>
@@ -552,6 +552,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
@@ -913,51 +914,131 @@
       <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="8"/>
-      <c r="Q8" s="8"/>
-      <c r="R8" s="8"/>
-      <c r="S8" s="8"/>
-      <c r="T8" s="8"/>
-      <c r="U8" s="8"/>
+      <c r="B8" s="7">
+        <v>2730</v>
+      </c>
+      <c r="C8" s="8">
+        <v>609</v>
+      </c>
+      <c r="D8" s="8">
+        <v>91.7</v>
+      </c>
+      <c r="E8" s="8">
+        <v>20.6</v>
+      </c>
+      <c r="F8" s="8">
+        <v>12</v>
+      </c>
+      <c r="G8" s="8">
+        <v>2.59</v>
+      </c>
+      <c r="H8" s="8">
+        <v>53.9</v>
+      </c>
+      <c r="I8" s="8">
+        <v>12</v>
+      </c>
+      <c r="J8" s="8">
+        <v>26.1</v>
+      </c>
+      <c r="K8" s="9">
+        <v>5.52</v>
+      </c>
+      <c r="L8" s="7">
+        <v>2940</v>
+      </c>
+      <c r="M8" s="8">
+        <v>167</v>
+      </c>
+      <c r="N8" s="8">
+        <v>98.8</v>
+      </c>
+      <c r="O8" s="8">
+        <v>2.96</v>
+      </c>
+      <c r="P8" s="8">
+        <v>12.9</v>
+      </c>
+      <c r="Q8" s="8">
+        <v>0.151</v>
+      </c>
+      <c r="R8" s="8">
+        <v>58</v>
+      </c>
+      <c r="S8" s="8">
+        <v>2.48</v>
+      </c>
+      <c r="T8" s="8">
+        <v>27.9</v>
+      </c>
+      <c r="U8" s="8">
+        <v>1.63</v>
+      </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="8"/>
-      <c r="N9" s="8"/>
-      <c r="O9" s="8"/>
-      <c r="P9" s="8"/>
-      <c r="Q9" s="8"/>
-      <c r="R9" s="8"/>
-      <c r="S9" s="8"/>
-      <c r="T9" s="8"/>
-      <c r="U9" s="8"/>
+      <c r="B9" s="7">
+        <v>2750</v>
+      </c>
+      <c r="C9" s="8">
+        <v>656</v>
+      </c>
+      <c r="D9" s="8">
+        <v>92.3</v>
+      </c>
+      <c r="E9" s="8">
+        <v>22.3</v>
+      </c>
+      <c r="F9" s="8">
+        <v>12</v>
+      </c>
+      <c r="G9" s="8">
+        <v>2.79</v>
+      </c>
+      <c r="H9" s="8">
+        <v>54.3</v>
+      </c>
+      <c r="I9" s="8">
+        <v>12.9</v>
+      </c>
+      <c r="J9" s="8">
+        <v>26.6</v>
+      </c>
+      <c r="K9" s="9">
+        <v>5.44</v>
+      </c>
+      <c r="L9" s="7">
+        <v>2980</v>
+      </c>
+      <c r="M9" s="8">
+        <v>173</v>
+      </c>
+      <c r="N9" s="8">
+        <v>100</v>
+      </c>
+      <c r="O9" s="8">
+        <v>3.14</v>
+      </c>
+      <c r="P9" s="8">
+        <v>13</v>
+      </c>
+      <c r="Q9" s="8">
+        <v>0.14499999999999999</v>
+      </c>
+      <c r="R9" s="8">
+        <v>58.9</v>
+      </c>
+      <c r="S9" s="8">
+        <v>2.64</v>
+      </c>
+      <c r="T9" s="8">
+        <v>28.3</v>
+      </c>
+      <c r="U9" s="8">
+        <v>1.58</v>
+      </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
@@ -1116,26 +1197,66 @@
       <c r="A13" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="8"/>
-      <c r="N13" s="8"/>
-      <c r="O13" s="8"/>
-      <c r="P13" s="8"/>
-      <c r="Q13" s="8"/>
-      <c r="R13" s="8"/>
-      <c r="S13" s="8"/>
-      <c r="T13" s="8"/>
-      <c r="U13" s="8"/>
+      <c r="B13" s="7">
+        <v>730</v>
+      </c>
+      <c r="C13" s="8">
+        <v>619</v>
+      </c>
+      <c r="D13" s="8">
+        <v>92.2</v>
+      </c>
+      <c r="E13" s="8">
+        <v>21</v>
+      </c>
+      <c r="F13" s="8">
+        <v>12</v>
+      </c>
+      <c r="G13" s="8">
+        <v>2.64</v>
+      </c>
+      <c r="H13" s="8">
+        <v>54.4</v>
+      </c>
+      <c r="I13" s="8">
+        <v>12.4</v>
+      </c>
+      <c r="J13" s="8">
+        <v>25.9</v>
+      </c>
+      <c r="K13" s="9">
+        <v>5.89</v>
+      </c>
+      <c r="L13" s="7">
+        <v>2940</v>
+      </c>
+      <c r="M13" s="8">
+        <v>165</v>
+      </c>
+      <c r="N13" s="8">
+        <v>99.6</v>
+      </c>
+      <c r="O13" s="8">
+        <v>3.11</v>
+      </c>
+      <c r="P13" s="8">
+        <v>12.9</v>
+      </c>
+      <c r="Q13" s="8">
+        <v>0.124</v>
+      </c>
+      <c r="R13" s="8">
+        <v>58.7</v>
+      </c>
+      <c r="S13" s="8">
+        <v>2.75</v>
+      </c>
+      <c r="T13" s="8">
+        <v>28</v>
+      </c>
+      <c r="U13" s="8">
+        <v>1.39</v>
+      </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>

</xml_diff>